<commit_message>
add dinning room asset
</commit_message>
<xml_diff>
--- a/Documentation/The Contradiction StoryBoard.xlsx
+++ b/Documentation/The Contradiction StoryBoard.xlsx
@@ -403,40 +403,40 @@
     <t xml:space="preserve">berjalan ke ujung lorong</t>
   </si>
   <si>
+    <t xml:space="preserve">taplak meja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bekerja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mendapatkan balasan dari samuel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ke tempat samuel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mengisi token</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tempat tisu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jangan mandi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jangan sarapan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lorong</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lampu plafon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jangan kerja</t>
+  </si>
+  <si>
     <t xml:space="preserve">belum dimulai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">taplak meja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bekerja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mendapatkan balasan dari samuel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ke tempat samuel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mengisi token</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tempat tisu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jangan mandi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jangan sarapan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lorong</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lampu plafon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jangan kerja</t>
   </si>
   <si>
     <t xml:space="preserve">jangan melihat pesan samuel</t>
@@ -1950,11 +1950,11 @@
         <v>126</v>
       </c>
       <c r="E68" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>127</v>
+        <v>9</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1965,20 +1965,20 @@
         <v>15</v>
       </c>
       <c r="E69" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C70" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>41</v>
       </c>
       <c r="E70" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1986,11 +1986,11 @@
         <v>85</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E71" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1998,11 +1998,11 @@
         <v>88</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E72" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2010,11 +2010,11 @@
         <v>90</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E73" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2022,11 +2022,11 @@
         <v>92</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E74" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2037,20 +2037,20 @@
         <v>126</v>
       </c>
       <c r="E75" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C76" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="D76" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="D76" s="4" t="s">
-        <v>134</v>
-      </c>
       <c r="E76" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2058,11 +2058,11 @@
         <v>68</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E77" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2070,20 +2070,20 @@
         <v>6</v>
       </c>
       <c r="B78" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C78" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="C78" s="4" t="s">
+      <c r="D78" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="D78" s="4" t="s">
+      <c r="E78" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="F78" s="4" t="s">
         <v>138</v>
-      </c>
-      <c r="E78" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="F78" s="4" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2164,7 +2164,7 @@
         <v>0</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2317,7 +2317,7 @@
         <v>0</v>
       </c>
       <c r="F96" s="4" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2578,7 +2578,7 @@
         <v>0</v>
       </c>
       <c r="F118" s="4" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2605,7 +2605,7 @@
         <v>0</v>
       </c>
       <c r="F120" s="4" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>